<commit_message>
Agregar tabla dinámica real + segmentador (paso 7)
- Inyecta partes OOXML construidas a mano: pivotCacheDefinition/Records,
  pivotTable (Categoria en filas, Mes en columnas, Suma de Total Venta),
  slicerCache y slicer por Producto, con su drawing.
- Conecta workbook (pivotCaches + extLst slicerCaches), worksheet
  (drawing + extLst slicerList), content-types y relationships.
- refreshOnLoad + fullCalcOnLoad para que Excel reconstruya la dinamica.
- Encabezados de tabla a una sola linea para que coincidan con los
  nombres de campo del cache.
- scripts/inject_pivot.py genera e inyecta estas partes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WaXhr28UL459jUkxGwVfpA
</commit_message>
<xml_diff>
--- a/Reporte_Ventas_Jhon_Martinez.xlsx
+++ b/Reporte_Ventas_Jhon_Martinez.xlsx
@@ -11,9 +11,20 @@
     <sheet name="Categorías" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Gráficos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Análisis" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TablaDinamica" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <pivotCaches>
+    <pivotCache cacheId="1" r:id="rId8"/>
+  </pivotCaches>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId9"/>
+      </x14:slicerCaches>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -510,6 +521,745 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" Requires="sle">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>8</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>18</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:to>
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Producto"/>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Producto"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback>
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>8</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>18</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2" name="Producto"/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-EC"/>
+                <a:t>Segmentador: Producto</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Fallback>
+  </mc:AlternateContent>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Excel" refreshedDate="46000" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="50" refreshOnLoad="1" saveData="1">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A5:H55" sheet="Ventas"/>
+  </cacheSource>
+  <cacheFields count="8">
+    <cacheField name="Mes" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Enero"/>
+        <s v="Febrero"/>
+        <s v="Marzo"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Producto" numFmtId="0">
+      <sharedItems count="10">
+        <s v="Impresora"/>
+        <s v="Toner"/>
+        <s v="Router"/>
+        <s v="Tinta"/>
+        <s v="Carpeta"/>
+        <s v="Lápiz"/>
+        <s v="Escritorio"/>
+        <s v="Calculadora"/>
+        <s v="Cuadernos"/>
+        <s v="Monitor"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Categoría" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Tecnología"/>
+        <s v="Papelería"/>
+        <s v="Oficina"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Cantidad Vendida" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="20"/>
+    </cacheField>
+    <cacheField name="Precio Unitario" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="5" maxValue="100"/>
+    </cacheField>
+    <cacheField name="Subtotal" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="10" maxValue="1300"/>
+    </cacheField>
+    <cacheField name="IVA" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.5" maxValue="195"/>
+    </cacheField>
+    <cacheField name="Total Venta" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="11.5" maxValue="1495"/>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="50">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="75"/>
+    <n v="750"/>
+    <n v="112.5"/>
+    <n v="862.5"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="11"/>
+    <n v="15"/>
+    <n v="165"/>
+    <n v="24.75"/>
+    <n v="189.75"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="11"/>
+    <n v="15"/>
+    <n v="165"/>
+    <n v="24.75"/>
+    <n v="189.75"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="15"/>
+    <n v="50"/>
+    <n v="750"/>
+    <n v="112.5"/>
+    <n v="862.5"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="18"/>
+    <n v="50"/>
+    <n v="900"/>
+    <n v="135"/>
+    <n v="1035"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="19"/>
+    <n v="10"/>
+    <n v="190"/>
+    <n v="28.5"/>
+    <n v="218.5"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="15"/>
+    <n v="5"/>
+    <n v="75"/>
+    <n v="11.25"/>
+    <n v="86.25"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="100"/>
+    <n v="100"/>
+    <n v="15"/>
+    <n v="115"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="9"/>
+    <n v="100"/>
+    <n v="900"/>
+    <n v="135"/>
+    <n v="1035"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="8"/>
+    <n v="75"/>
+    <n v="600"/>
+    <n v="90"/>
+    <n v="690"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="75"/>
+    <n v="375"/>
+    <n v="56.25"/>
+    <n v="431.25"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="16"/>
+    <n v="75"/>
+    <n v="1200"/>
+    <n v="180"/>
+    <n v="1380"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="7"/>
+    <x v="0"/>
+    <n v="13"/>
+    <n v="50"/>
+    <n v="650"/>
+    <n v="97.5"/>
+    <n v="747.5"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="9"/>
+    <n v="15"/>
+    <n v="135"/>
+    <n v="20.25"/>
+    <n v="155.25"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="17"/>
+    <n v="75"/>
+    <n v="1275"/>
+    <n v="191.25"/>
+    <n v="1466.25"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="7"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="5"/>
+    <n v="50"/>
+    <n v="7.5"/>
+    <n v="57.5"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="7"/>
+    <x v="0"/>
+    <n v="20"/>
+    <n v="5"/>
+    <n v="100"/>
+    <n v="15"/>
+    <n v="115"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="13"/>
+    <n v="25"/>
+    <n v="325"/>
+    <n v="48.75"/>
+    <n v="373.75"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="20"/>
+    <n v="20"/>
+    <n v="3"/>
+    <n v="23"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="12"/>
+    <n v="25"/>
+    <n v="300"/>
+    <n v="45"/>
+    <n v="345"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="16"/>
+    <n v="20"/>
+    <n v="320"/>
+    <n v="48"/>
+    <n v="368"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="20"/>
+    <n v="20"/>
+    <n v="400"/>
+    <n v="60"/>
+    <n v="460"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="15"/>
+    <n v="20"/>
+    <n v="300"/>
+    <n v="45"/>
+    <n v="345"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="14"/>
+    <n v="50"/>
+    <n v="700"/>
+    <n v="105"/>
+    <n v="805"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="14"/>
+    <n v="50"/>
+    <n v="700"/>
+    <n v="105"/>
+    <n v="805"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="18"/>
+    <n v="10"/>
+    <n v="180"/>
+    <n v="27"/>
+    <n v="207"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="2"/>
+    <n v="10"/>
+    <n v="20"/>
+    <n v="3"/>
+    <n v="23"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="12"/>
+    <n v="100"/>
+    <n v="1200"/>
+    <n v="180"/>
+    <n v="1380"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="19"/>
+    <n v="15"/>
+    <n v="285"/>
+    <n v="42.75"/>
+    <n v="327.75"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="9"/>
+    <n v="50"/>
+    <n v="450"/>
+    <n v="67.5"/>
+    <n v="517.5"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="2"/>
+    <n v="15"/>
+    <n v="30"/>
+    <n v="4.5"/>
+    <n v="34.5"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="3"/>
+    <n v="20"/>
+    <n v="60"/>
+    <n v="9"/>
+    <n v="69"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="9"/>
+    <n v="15"/>
+    <n v="135"/>
+    <n v="20.25"/>
+    <n v="155.25"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="1"/>
+    <n v="25"/>
+    <n v="25"/>
+    <n v="3.75"/>
+    <n v="28.75"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="13"/>
+    <n v="100"/>
+    <n v="1300"/>
+    <n v="195"/>
+    <n v="1495"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="3"/>
+    <n v="5"/>
+    <n v="15"/>
+    <n v="2.25"/>
+    <n v="17.25"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="9"/>
+    <n v="15"/>
+    <n v="135"/>
+    <n v="20.25"/>
+    <n v="155.25"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="15"/>
+    <n v="20"/>
+    <n v="300"/>
+    <n v="45"/>
+    <n v="345"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="9"/>
+    <n v="15"/>
+    <n v="135"/>
+    <n v="20.25"/>
+    <n v="155.25"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="2"/>
+    <n v="5"/>
+    <n v="10"/>
+    <n v="1.5"/>
+    <n v="11.5"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="12"/>
+    <n v="25"/>
+    <n v="300"/>
+    <n v="45"/>
+    <n v="345"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="10"/>
+    <n v="50"/>
+    <n v="7.5"/>
+    <n v="57.5"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="14"/>
+    <n v="75"/>
+    <n v="1050"/>
+    <n v="157.5"/>
+    <n v="1207.5"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="5"/>
+    <n v="5"/>
+    <n v="25"/>
+    <n v="3.75"/>
+    <n v="28.75"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="7"/>
+    <n v="5"/>
+    <n v="35"/>
+    <n v="5.25"/>
+    <n v="40.25"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="50"/>
+    <n v="500"/>
+    <n v="75"/>
+    <n v="575"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="19"/>
+    <n v="10"/>
+    <n v="190"/>
+    <n v="28.5"/>
+    <n v="218.5"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="12"/>
+    <n v="10"/>
+    <n v="120"/>
+    <n v="18"/>
+    <n v="138"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="10"/>
+    <n v="20"/>
+    <n v="200"/>
+    <n v="30"/>
+    <n v="230"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="2"/>
+    <n v="10"/>
+    <n v="20"/>
+    <n v="3"/>
+    <n v="23"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinamica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A4:E9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de Total Venta" fld="7" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slicer_Producto" sourceName="Producto">
+  <pivotTables>
+    <pivotTable tabId="5" name="TablaDinamica1"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1">
+      <items count="10">
+        <i x="0"/>
+        <i x="1"/>
+        <i x="2"/>
+        <i x="3"/>
+        <i x="4"/>
+        <i x="5"/>
+        <i x="6"/>
+        <i x="7"/>
+        <i x="8"/>
+        <i x="9"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <slicer name="Producto" cache="Slicer_Producto" caption="Producto" startItem="0" columnCount="1" showCaption="1" level="0" style="SlicerStyleLight1" rowHeight="241300"/>
+</slicers>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -861,14 +1611,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Cantidad
-Vendida</t>
+          <t>Cantidad Vendida</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Precio
-Unitario</t>
+          <t>Precio Unitario</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -883,8 +1631,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Total
-Venta</t>
+          <t>Total Venta</t>
         </is>
       </c>
     </row>
@@ -3007,4 +3754,47 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>TABLA DINÁMICA – Ventas por Categoría y Mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>Segmentador (slicer) por Producto a la derecha →</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId3"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>